<commit_message>
Add PO numbers and confirm order 1 date
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z5pCoVvnUESSHvBHrad3z
</commit_message>
<xml_diff>
--- a/tracker/Filter_Order_Log.xlsx
+++ b/tracker/Filter_Order_Log.xlsx
@@ -607,7 +607,11 @@
           <t>766028</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>380118</t>
+        </is>
+      </c>
       <c r="F8" t="n">
         <v>8</v>
       </c>
@@ -637,7 +641,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Urgent, units unknown at time of order. Email request was 9/25, receipt dated 9/22 - confirm date.</t>
+          <t>Urgent, units unknown at time of order.</t>
         </is>
       </c>
     </row>
@@ -662,7 +666,11 @@
           <t>766028</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>380118</t>
+        </is>
+      </c>
       <c r="F9" t="n">
         <v>8</v>
       </c>
@@ -705,7 +713,11 @@
           <t>770738</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>382244</t>
+        </is>
+      </c>
       <c r="F10" t="n">
         <v>8</v>
       </c>
@@ -760,7 +772,11 @@
           <t>770738</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>382244</t>
+        </is>
+      </c>
       <c r="F11" t="n">
         <v>8</v>
       </c>
@@ -803,7 +819,11 @@
           <t>770738</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>382244</t>
+        </is>
+      </c>
       <c r="F12" t="n">
         <v>8</v>
       </c>
@@ -846,7 +866,11 @@
           <t>770738</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>382244</t>
+        </is>
+      </c>
       <c r="F13" t="n">
         <v>8</v>
       </c>

</xml_diff>